<commit_message>
pivot les sl drop bar
</commit_message>
<xml_diff>
--- a/data/gravel/Argon 18 Dark Matter 2025.xlsx
+++ b/data/gravel/Argon 18 Dark Matter 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/walker/Documents/Github/Bike Geometry Project/data/gravel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC893F3-0A85-1C4D-95AC-F23EDEC30B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833892AB-AA63-0E4F-9E80-86AEE159E28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30480" yWindow="-28300" windowWidth="33620" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27620" yWindow="-28300" windowWidth="33620" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1139,7 +1139,7 @@
         <v>27</v>
       </c>
       <c r="C12">
-        <f t="shared" ref="C10:C27" si="2">K12*10</f>
+        <f t="shared" ref="C12:C27" si="2">K12*10</f>
         <v>507</v>
       </c>
       <c r="D12">

</xml_diff>